<commit_message>
fix(inventory-ledger): V1 定向修复 6 项(基于 2b1be80 内容)
1. 同采购单多张费用单: 分摊额改累计写入, 防覆盖少计; 结账核对改期间级汇总
2. 费用分摊限定关联采购同月, 跨期/已结账期间分摊拒绝(E09/E15)
3. 采购成本更正行继承原行附加费用分摊额, 费用不丢失
4. 导入: 来源行号随行保留(fee/opening 同修); 业务写入+导入登记+审计
   放入 store.batch() 原子提交, 中途失败整批不落盘
5. 加权成本内部全精度均价: 期末=round2(期末池数量×内部均价), 出库=池−期末
   守恒恒等; 大数量/循环小数单价/零结存不再误报 E06/E07
6. 新增 tests/test_v1_fixes.py 五组回归; AC8 尾差测试改为守恒断言
   保留 AC1-AC8, 全文 46 passed
</commit_message>
<xml_diff>
--- a/inventory-ledger-skill/examples/demo/output/进销存台账.xlsx
+++ b/inventory-ledger-skill/examples/demo/output/进销存台账.xlsx
@@ -453,7 +453,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>eed13d0a8e15</t>
+          <t>a70114b0e4fd</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:41</t>
+          <t>2026-10-27 19:37:28</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>19</t>
         </is>
       </c>
     </row>
@@ -729,6 +729,11 @@
           <t>CSV</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
           <t>b9f3ba3b634a63898b45072d300b5e5be402e358c8c85954973025274e0c75e6</t>
@@ -736,12 +741,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>B20261027174443</t>
+          <t>B20261027193730</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:43</t>
+          <t>2026-10-27 19:37:30</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -928,7 +933,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:44</t>
+          <t>2026-10-27 19:37:30</t>
         </is>
       </c>
     </row>
@@ -976,10 +981,10 @@
         <v>75</v>
       </c>
       <c r="N3" t="n">
-        <v>824.09</v>
+        <v>824.08</v>
       </c>
       <c r="O3" t="n">
-        <v>770.91</v>
+        <v>770.92</v>
       </c>
       <c r="P3" t="n">
         <v>5.3167</v>
@@ -994,7 +999,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:44</t>
+          <t>2026-10-27 19:37:30</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1052,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:44</t>
+          <t>2026-10-27 19:37:30</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1105,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:44</t>
+          <t>2026-10-27 19:37:30</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1158,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:44</t>
+          <t>2026-10-27 19:37:30</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1225,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:45</t>
+          <t>2026-10-27 19:37:31</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1265,7 @@
         <v>145</v>
       </c>
       <c r="K8" t="n">
-        <v>770.91</v>
+        <v>770.92</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
@@ -1272,10 +1277,10 @@
         <v>0</v>
       </c>
       <c r="O8" t="n">
-        <v>770.91</v>
+        <v>770.92</v>
       </c>
       <c r="P8" t="n">
-        <v>5.3166</v>
+        <v>5.3167</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1287,7 +1292,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:45</t>
+          <t>2026-10-27 19:37:31</t>
         </is>
       </c>
     </row>
@@ -1346,7 +1351,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:45</t>
+          <t>2026-10-27 19:37:31</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1410,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:45</t>
+          <t>2026-10-27 19:37:31</t>
         </is>
       </c>
     </row>
@@ -1464,7 +1469,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:45</t>
+          <t>2026-10-27 19:37:31</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1537,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:41</t>
+          <t>2026-10-27 19:37:28</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1574,7 +1579,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:41</t>
+          <t>2026-10-27 19:37:28</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1611,7 +1616,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:41</t>
+          <t>2026-10-27 19:37:28</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1648,7 +1653,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:28</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1685,7 +1690,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:28</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1722,7 +1727,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1764,7 +1769,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1784,12 +1789,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认期初; 批次: B20261027174442-000001</t>
+          <t>用户确认: 用户确认期初; 批次: B20261027193729-000001</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>B20261027174442-000001</t>
+          <t>B20261027193729-000001</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1806,7 +1811,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1843,7 +1848,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1863,12 +1868,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认采购; 批次: B20261027174442-000002</t>
+          <t>用户确认: 用户确认采购; 批次: B20261027193729-000002</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>B20261027174442-000002</t>
+          <t>B20261027193729-000002</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1885,7 +1890,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1922,7 +1927,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1942,12 +1947,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认采购; 批次: B20261027174442-000003</t>
+          <t>用户确认: 用户确认采购; 批次: B20261027193729-000003</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>B20261027174442-000003</t>
+          <t>B20261027193729-000003</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1964,7 +1969,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1989,7 +1994,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>批次:B20261027174442</t>
+          <t>批次:B20261027193729</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2006,7 +2011,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2026,12 +2031,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认销售; 批次: B20261027174442-000004</t>
+          <t>用户确认: 用户确认销售; 批次: B20261027193729-000004</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>B20261027174442-000004</t>
+          <t>B20261027193729-000004</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2048,7 +2053,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:43</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2073,7 +2078,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>批次:B20261027174443</t>
+          <t>批次:B20261027193729</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2090,7 +2095,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:43</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2110,12 +2115,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认销售; 批次: B20261027174443-000005</t>
+          <t>用户确认: 用户确认销售; 批次: B20261027193729-000005</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>B20261027174443-000005</t>
+          <t>B20261027193729-000005</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2132,7 +2137,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:43</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2157,7 +2162,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>批次:B20261027174443</t>
+          <t>批次:B20261027193729</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2174,7 +2179,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:43</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2194,12 +2199,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认调拨; 批次: B20261027174443-000006</t>
+          <t>用户确认: 用户确认调拨; 批次: B20261027193729-000006</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>B20261027174443-000006</t>
+          <t>B20261027193729-000006</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2216,7 +2221,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:43</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2241,7 +2246,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>批次:B20261027174443</t>
+          <t>批次:B20261027193729</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2258,7 +2263,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:43</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2278,12 +2283,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认调整; 批次: B20261027174443-000007</t>
+          <t>用户确认: 用户确认调整; 批次: B20261027193729-000007</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>B20261027174443-000007</t>
+          <t>B20261027193729-000007</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2300,7 +2305,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:43</t>
+          <t>2026-10-27 19:37:30</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2337,7 +2342,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:43</t>
+          <t>2026-10-27 19:37:30</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2357,12 +2362,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认费用; 批次: B20261027174443-000008</t>
+          <t>用户确认: 用户确认费用; 批次: B20261027193730-000008</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>B20261027174443-000008</t>
+          <t>B20261027193730-000008</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2379,7 +2384,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:43</t>
+          <t>2026-10-27 19:37:30</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2421,7 +2426,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:44</t>
+          <t>2026-10-27 19:37:30</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2463,7 +2468,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:44</t>
+          <t>2026-10-27 19:37:31</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2500,7 +2505,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:44</t>
+          <t>2026-10-27 19:37:31</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2537,7 +2542,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:44</t>
+          <t>2026-10-27 19:37:31</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2557,12 +2562,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认采购; 批次: B20261027174444-000009</t>
+          <t>用户确认: 用户确认采购; 批次: B20261027193731-000009</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>B20261027174444-000009</t>
+          <t>B20261027193731-000009</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2579,7 +2584,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:44</t>
+          <t>2026-10-27 19:37:31</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2604,7 +2609,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>批次:B20261027174444</t>
+          <t>批次:B20261027193731</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2621,7 +2626,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:44</t>
+          <t>2026-10-27 19:37:31</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2641,12 +2646,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认销售; 批次: B20261027174444-000010</t>
+          <t>用户确认: 用户确认销售; 批次: B20261027193731-000010</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>B20261027174444-000010</t>
+          <t>B20261027193731-000010</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2663,7 +2668,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:45</t>
+          <t>2026-10-27 19:37:31</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2781,7 +2786,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>B20261027174442-000001</t>
+          <t>B20261027193729-000001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2813,7 +2818,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -2835,7 +2840,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>B20261027174442-000002</t>
+          <t>B20261027193729-000002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2867,7 +2872,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -2889,7 +2894,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>B20261027174442-000003</t>
+          <t>B20261027193729-000003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2921,7 +2926,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -2943,7 +2948,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>B20261027174442-000004</t>
+          <t>B20261027193729-000004</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2975,7 +2980,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -2997,7 +3002,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>B20261027174443-000005</t>
+          <t>B20261027193729-000005</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3029,7 +3034,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:43</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -3051,7 +3056,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>B20261027174443-000006</t>
+          <t>B20261027193729-000006</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3083,7 +3088,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:43</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -3105,7 +3110,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>B20261027174443-000007</t>
+          <t>B20261027193729-000007</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3137,7 +3142,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:43</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -3159,7 +3164,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>B20261027174443-000008</t>
+          <t>B20261027193730-000008</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -3191,7 +3196,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:43</t>
+          <t>2026-10-27 19:37:30</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -3213,7 +3218,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>B20261027174444-000009</t>
+          <t>B20261027193731-000009</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3245,7 +3250,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:44</t>
+          <t>2026-10-27 19:37:31</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -3267,7 +3272,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>B20261027174444-000010</t>
+          <t>B20261027193731-000010</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3299,7 +3304,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:44</t>
+          <t>2026-10-27 19:37:31</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -3375,7 +3380,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:44</t>
+          <t>2026-10-27 19:37:30</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -3405,7 +3410,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:45</t>
+          <t>2026-10-27 19:37:31</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -3488,7 +3493,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:41</t>
+          <t>2026-10-27 19:37:28</t>
         </is>
       </c>
     </row>
@@ -3515,7 +3520,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:41</t>
+          <t>2026-10-27 19:37:28</t>
         </is>
       </c>
     </row>
@@ -3578,7 +3583,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:28</t>
         </is>
       </c>
     </row>
@@ -3600,7 +3605,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:28</t>
         </is>
       </c>
     </row>
@@ -3750,6 +3755,11 @@
           <t>CSV</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr">
         <is>
           <t>a8877ed7b01f190bb076bcc7468ce82931eda30e5cc50cd54f4b01ef7b2dcf89</t>
@@ -3757,12 +3767,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>B20261027174442</t>
+          <t>B20261027193729</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -3821,6 +3831,11 @@
           <t>CSV</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>a8877ed7b01f190bb076bcc7468ce82931eda30e5cc50cd54f4b01ef7b2dcf89</t>
@@ -3828,12 +3843,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>B20261027174442</t>
+          <t>B20261027193729</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -3892,6 +3907,11 @@
           <t>CSV</t>
         </is>
       </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>a8877ed7b01f190bb076bcc7468ce82931eda30e5cc50cd54f4b01ef7b2dcf89</t>
@@ -3899,12 +3919,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>B20261027174442</t>
+          <t>B20261027193729</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -4137,6 +4157,11 @@
           <t>CSV</t>
         </is>
       </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr">
         <is>
           <t>4880c3cd6fbd05a7c9e3551925ca14a522a1c43a93edf8b1322fd5beb99e3a70</t>
@@ -4144,12 +4169,12 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>B20261027174442</t>
+          <t>B20261027193729</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -4231,6 +4256,11 @@
           <t>CSV</t>
         </is>
       </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="V3" t="inlineStr">
         <is>
           <t>4880c3cd6fbd05a7c9e3551925ca14a522a1c43a93edf8b1322fd5beb99e3a70</t>
@@ -4238,12 +4268,12 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>B20261027174442</t>
+          <t>B20261027193729</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -4325,6 +4355,11 @@
           <t>CSV</t>
         </is>
       </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr">
         <is>
           <t>9a74f82a530349488a340b6612620c36b3ac7d7458daef4d08ff1685d36aed48</t>
@@ -4332,12 +4367,12 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>B20261027174442</t>
+          <t>B20261027193729</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -4419,6 +4454,11 @@
           <t>CSV</t>
         </is>
       </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr">
         <is>
           <t>af5bebae5b820e181409c37d127d99208cc597735eceaf163eb9b198ea1d7d70</t>
@@ -4426,12 +4466,12 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>B20261027174444</t>
+          <t>B20261027193731</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:44</t>
+          <t>2026-10-27 19:37:31</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -4680,6 +4720,11 @@
           <t>CSV</t>
         </is>
       </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="W2" t="inlineStr">
         <is>
           <t>4c3be387aeba8a135d45bd4191b2e6f4ca66fa80577731290d50a1c71c2503b6</t>
@@ -4687,12 +4732,12 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>B20261027174442</t>
+          <t>B20261027193729</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -4768,7 +4813,7 @@
         <v>8</v>
       </c>
       <c r="Q3" t="n">
-        <v>797.51</v>
+        <v>797.5</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -4785,6 +4830,11 @@
           <t>CSV</t>
         </is>
       </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="W3" t="inlineStr">
         <is>
           <t>4c3be387aeba8a135d45bd4191b2e6f4ca66fa80577731290d50a1c71c2503b6</t>
@@ -4792,12 +4842,12 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>B20261027174442</t>
+          <t>B20261027193729</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:42</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -4890,6 +4940,11 @@
           <t>CSV</t>
         </is>
       </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="W4" t="inlineStr">
         <is>
           <t>405c22439c9567ccee51d5e70f32c8b8b8ed94e3f0010f70ec4b459e6cf25923</t>
@@ -4897,12 +4952,12 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>B20261027174443</t>
+          <t>B20261027193729</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:43</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
@@ -4995,6 +5050,11 @@
           <t>CSV</t>
         </is>
       </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="W5" t="inlineStr">
         <is>
           <t>6d2c3c5c3018f7584ef49f5982e43f411c5a3b122b8b8507cb340de6b836dfc2</t>
@@ -5002,12 +5062,12 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>B20261027174444</t>
+          <t>B20261027193731</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:44</t>
+          <t>2026-10-27 19:37:31</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
@@ -5196,6 +5256,11 @@
           <t>CSV</t>
         </is>
       </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="O2" t="inlineStr">
         <is>
           <t>24776315d207fd2cec81bd9cc06b8eccced78a0c3e25cf7b1a3696c407c62e3e</t>
@@ -5203,12 +5268,12 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>B20261027174443</t>
+          <t>B20261027193729</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:43</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -5412,6 +5477,11 @@
           <t>CSV</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R2" t="inlineStr">
         <is>
           <t>92dbbc1492b6e4ace4014abeca235229dd14c690bb2396bef2510f4d04ceb75e</t>
@@ -5419,12 +5489,12 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>B20261027174443</t>
+          <t>B20261027193729</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-10-27 17:44:43</t>
+          <t>2026-10-27 19:37:29</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">

</xml_diff>

<commit_message>
fix(inventory-ledger): V1 数据完整性收口(数据完整性 Fix1-3)
Fix1 批次内部重复业务行防重: add_purchases/add_sales 规范化后行间指纹互查,
importer.preview 同批次互查(预览与提交一致); 采购+销售, E12, 默认整批拒绝;
指纹组合沿用 期间+单号+明细行号+SKU+仓库, 未重新定义单据唯一性。

Fix2 费用登记前验证关联采购单: add_fee/_normalize_fee 登记阶段即要求
关联采购单在同月存在有效入库行(E16), 杜绝"已登记、无法分摊、无法结账"
的跨期悬挂; 已结账期间 E15 不变; 同单多费累计分摊不变。

Fix3 统一导入批次号: Store.next_batch_id() 唯一确定(时间戳+导入序号),
业务行"导入批次"/导入登记"批次号"/审计引用同一 ID, 生成与使用均纳入
Store.batch() 原子提交; register_import 接受 batch 参数并兼容旧调用。

新增 tests/test_data_integrity.py(11 项), 更新 test_v1_fixes 跨期费用场景
(登记阶段拒绝), 全量 57 passed; demo 两月结账数字与基线一致;
git diff --check 干净; README/workflows 同步。独立验收 PASS。
</commit_message>
<xml_diff>
--- a/inventory-ledger-skill/examples/demo/output/进销存台账.xlsx
+++ b/inventory-ledger-skill/examples/demo/output/进销存台账.xlsx
@@ -453,7 +453,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>a70114b0e4fd</t>
+          <t>0e6a918a4558</t>
         </is>
       </c>
     </row>
@@ -573,7 +573,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:28</t>
+          <t>2026-10-27 20:33:40</t>
         </is>
       </c>
     </row>
@@ -741,12 +741,12 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>B20261027193730</t>
+          <t>B20261027203342-000008</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:30</t>
+          <t>2026-10-27 20:33:42</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -933,7 +933,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:30</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
     </row>
@@ -999,7 +999,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:30</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:30</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
     </row>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:30</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:30</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:31</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
     </row>
@@ -1292,7 +1292,7 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:31</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:31</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1410,7 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:31</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
     </row>
@@ -1469,7 +1469,7 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:31</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1537,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:28</t>
+          <t>2026-10-27 20:33:40</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1579,7 +1579,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:28</t>
+          <t>2026-10-27 20:33:40</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:28</t>
+          <t>2026-10-27 20:33:40</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1653,7 +1653,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:28</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:28</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1769,7 +1769,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1789,12 +1789,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认期初; 批次: B20261027193729-000001</t>
+          <t>用户确认: 用户确认期初; 批次: B20261027203341-000001</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>B20261027193729-000001</t>
+          <t>B20261027203341-000001</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1811,7 +1811,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1848,7 +1848,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1868,12 +1868,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认采购; 批次: B20261027193729-000002</t>
+          <t>用户确认: 用户确认采购; 批次: B20261027203341-000002</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>B20261027193729-000002</t>
+          <t>B20261027203341-000002</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1890,7 +1890,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1927,7 +1927,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1947,12 +1947,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认采购; 批次: B20261027193729-000003</t>
+          <t>用户确认: 用户确认采购; 批次: B20261027203341-000003</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>B20261027193729-000003</t>
+          <t>B20261027203341-000003</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>批次:B20261027193729</t>
+          <t>批次:B20261027203341-000004</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2031,12 +2031,12 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认销售; 批次: B20261027193729-000004</t>
+          <t>用户确认: 用户确认销售; 批次: B20261027203341-000004</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>B20261027193729-000004</t>
+          <t>B20261027203341-000004</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:42</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>批次:B20261027193729</t>
+          <t>批次:B20261027203342-000005</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:42</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2115,12 +2115,12 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认销售; 批次: B20261027193729-000005</t>
+          <t>用户确认: 用户确认销售; 批次: B20261027203342-000005</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>B20261027193729-000005</t>
+          <t>B20261027203342-000005</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:42</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2162,7 +2162,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>批次:B20261027193729</t>
+          <t>批次:B20261027203342-000006</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2179,7 +2179,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:42</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2199,12 +2199,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认调拨; 批次: B20261027193729-000006</t>
+          <t>用户确认: 用户确认调拨; 批次: B20261027203342-000006</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>B20261027193729-000006</t>
+          <t>B20261027203342-000006</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2221,7 +2221,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:42</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>批次:B20261027193729</t>
+          <t>批次:B20261027203342-000007</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2263,7 +2263,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:42</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2283,12 +2283,12 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认调整; 批次: B20261027193729-000007</t>
+          <t>用户确认: 用户确认调整; 批次: B20261027203342-000007</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>B20261027193729-000007</t>
+          <t>B20261027203342-000007</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2305,7 +2305,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:30</t>
+          <t>2026-10-27 20:33:42</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:30</t>
+          <t>2026-10-27 20:33:42</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2362,12 +2362,12 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认费用; 批次: B20261027193730-000008</t>
+          <t>用户确认: 用户确认费用; 批次: B20261027203342-000008</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>B20261027193730-000008</t>
+          <t>B20261027203342-000008</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:30</t>
+          <t>2026-10-27 20:33:42</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2426,7 +2426,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:30</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2468,7 +2468,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:31</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2505,7 +2505,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:31</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:31</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2562,12 +2562,12 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认采购; 批次: B20261027193731-000009</t>
+          <t>用户确认: 用户确认采购; 批次: B20261027203343-000009</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>B20261027193731-000009</t>
+          <t>B20261027203343-000009</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2584,7 +2584,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:31</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2609,7 +2609,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>批次:B20261027193731</t>
+          <t>批次:B20261027203343-000010</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:31</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2646,12 +2646,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>用户确认: 用户确认销售; 批次: B20261027193731-000010</t>
+          <t>用户确认: 用户确认销售; 批次: B20261027203343-000010</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>B20261027193731-000010</t>
+          <t>B20261027203343-000010</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2668,7 +2668,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:31</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2786,7 +2786,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>B20261027193729-000001</t>
+          <t>B20261027203341-000001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -2818,7 +2818,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -2840,7 +2840,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>B20261027193729-000002</t>
+          <t>B20261027203341-000002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2872,7 +2872,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -2894,7 +2894,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>B20261027193729-000003</t>
+          <t>B20261027203341-000003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2926,7 +2926,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -2948,7 +2948,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>B20261027193729-000004</t>
+          <t>B20261027203341-000004</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -3002,7 +3002,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>B20261027193729-000005</t>
+          <t>B20261027203342-000005</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3034,7 +3034,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:42</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -3056,7 +3056,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>B20261027193729-000006</t>
+          <t>B20261027203342-000006</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:42</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -3110,7 +3110,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>B20261027193729-000007</t>
+          <t>B20261027203342-000007</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:42</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -3164,7 +3164,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>B20261027193730-000008</t>
+          <t>B20261027203342-000008</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -3196,7 +3196,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:30</t>
+          <t>2026-10-27 20:33:42</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -3218,7 +3218,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>B20261027193731-000009</t>
+          <t>B20261027203343-000009</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3250,7 +3250,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:31</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -3272,7 +3272,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>B20261027193731-000010</t>
+          <t>B20261027203343-000010</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3304,7 +3304,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:31</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:30</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -3410,7 +3410,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:31</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -3493,7 +3493,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:28</t>
+          <t>2026-10-27 20:33:40</t>
         </is>
       </c>
     </row>
@@ -3520,7 +3520,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:28</t>
+          <t>2026-10-27 20:33:40</t>
         </is>
       </c>
     </row>
@@ -3583,7 +3583,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:28</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:28</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
     </row>
@@ -3767,12 +3767,12 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>B20261027193729</t>
+          <t>B20261027203341-000001</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -3843,12 +3843,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>B20261027193729</t>
+          <t>B20261027203341-000001</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -3919,12 +3919,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>B20261027193729</t>
+          <t>B20261027203341-000001</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -4169,12 +4169,12 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>B20261027193729</t>
+          <t>B20261027203341-000002</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
@@ -4268,12 +4268,12 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>B20261027193729</t>
+          <t>B20261027203341-000002</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -4367,12 +4367,12 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>B20261027193729</t>
+          <t>B20261027203341-000003</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -4466,12 +4466,12 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>B20261027193731</t>
+          <t>B20261027203343-000009</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:31</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
@@ -4732,12 +4732,12 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
-          <t>B20261027193729</t>
+          <t>B20261027203341-000004</t>
         </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
@@ -4842,12 +4842,12 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>B20261027193729</t>
+          <t>B20261027203341-000004</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:41</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -4952,12 +4952,12 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>B20261027193729</t>
+          <t>B20261027203342-000005</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:42</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr">
@@ -5062,12 +5062,12 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
-          <t>B20261027193731</t>
+          <t>B20261027203343-000010</t>
         </is>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:31</t>
+          <t>2026-10-27 20:33:43</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr">
@@ -5268,12 +5268,12 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>B20261027193729</t>
+          <t>B20261027203342-000006</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:42</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -5489,12 +5489,12 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>B20261027193729</t>
+          <t>B20261027203342-000007</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-10-27 19:37:29</t>
+          <t>2026-10-27 20:33:42</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">

</xml_diff>